<commit_message>
Final version - old baselines though
</commit_message>
<xml_diff>
--- a/assets/SciClaimEval26_Results.xlsx
+++ b/assets/SciClaimEval26_Results.xlsx
@@ -5,13 +5,15 @@
   <sheets>
     <sheet state="visible" name="Run Evaluations" sheetId="1" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Run Evaluations'!$A$1:$W$195</definedName>
+  </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1746" uniqueCount="605">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1836" uniqueCount="625">
   <si>
     <t>run_id</t>
   </si>
@@ -1832,6 +1834,66 @@
   </si>
   <si>
     <t>task1_routed_gptfable_SUBMIT</t>
+  </si>
+  <si>
+    <t>107fcb2da277a9ef2c526b8e265519ac</t>
+  </si>
+  <si>
+    <t>c0fb6fb246183c26400846a6656f2e0e</t>
+  </si>
+  <si>
+    <t>c1827e6c87b9a63f1d4e94ab9e9d70ea</t>
+  </si>
+  <si>
+    <t>fca8b45e3cc41568c3431721504e1bae</t>
+  </si>
+  <si>
+    <t>51744d10e0fca05a8dc564292920d5ab</t>
+  </si>
+  <si>
+    <t>4753ecef98b994f160bd27bccba435c4</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1IgkG9k5jrd4bNPie9IXTerex-UnRnliD</t>
+  </si>
+  <si>
+    <t>Claude Fable 5 (PNG-only)</t>
+  </si>
+  <si>
+    <t>b5684ef7e9b3f054fcf66f8cc4f04577</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1abF4tMdtqA4Y5szJYrHoAWo8U7JkTW9l</t>
+  </si>
+  <si>
+    <t>routed ensemble + GPT-5.5 + pair prior (PNG-only, leak-free)</t>
+  </si>
+  <si>
+    <t>a184f4b6fde90fa4d3e80cabf5fa83d8</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1LnDVc7K5xQ81xuMwB6QrkhZUc5lIxqQQ</t>
+  </si>
+  <si>
+    <t>routed ensemble + GPT-5.5 + Claude Fable 5 + pair prior (PNG-only, leak-free)</t>
+  </si>
+  <si>
+    <t>fd0f6d66d0d1d3cd9fe4daa782bee6c9</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=19VIoDpOhxPBzmxLfcglZqTqvRfOUdVSn</t>
+  </si>
+  <si>
+    <t>GPT 5.6 Sol</t>
+  </si>
+  <si>
+    <t>8104ad3204c680583aca8f143f0f9678</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=16AE02HDl_qEQihsAS-KSibJ4gOpwFR5p</t>
+  </si>
+  <si>
+    <t>routed ensemble + GPT-5.5 + Claude Fable 5 + GPT-5.6 Sol + pair prior (PNG-only, leak-free)</t>
   </si>
 </sst>
 </file>
@@ -1995,7 +2057,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:W185" displayName="SciClaimEval26_Results" name="SciClaimEval26_Results" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:W195" displayName="SciClaimEval26_Results" name="SciClaimEval26_Results" id="1">
+  <autoFilter ref="$A$1:$W$195"/>
   <tableColumns count="23">
     <tableColumn name="run_id" id="1"/>
     <tableColumn name="timestamp" id="2"/>
@@ -14355,30 +14418,68 @@
       <c r="AE185" s="6"/>
       <c r="AF185" s="6"/>
     </row>
-    <row r="186">
-      <c r="A186" s="12"/>
-      <c r="B186" s="6"/>
-      <c r="C186" s="6"/>
-      <c r="D186" s="6"/>
-      <c r="E186" s="6"/>
-      <c r="F186" s="12"/>
-      <c r="G186" s="12"/>
-      <c r="H186" s="12"/>
-      <c r="I186" s="13"/>
-      <c r="J186" s="13"/>
-      <c r="K186" s="13"/>
-      <c r="L186" s="13"/>
-      <c r="M186" s="13"/>
-      <c r="N186" s="13"/>
-      <c r="O186" s="13"/>
-      <c r="P186" s="13"/>
-      <c r="Q186" s="13"/>
-      <c r="R186" s="6"/>
-      <c r="S186" s="6"/>
-      <c r="T186" s="6"/>
-      <c r="U186" s="6"/>
-      <c r="V186" s="6"/>
-      <c r="W186" s="6"/>
+    <row r="186" ht="22.5" customHeight="1">
+      <c r="A186" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="B186" s="8">
+        <v>46202.85901620371</v>
+      </c>
+      <c r="C186" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D186" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E186" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F186" s="10" t="s">
+        <v>591</v>
+      </c>
+      <c r="G186" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H186" s="7" t="s">
+        <v>592</v>
+      </c>
+      <c r="I186" s="3">
+        <v>97.37</v>
+      </c>
+      <c r="J186" s="3">
+        <v>97.33</v>
+      </c>
+      <c r="K186" s="3">
+        <v>97.35</v>
+      </c>
+      <c r="L186" s="3">
+        <v>97.35</v>
+      </c>
+      <c r="M186" s="3">
+        <v>97.69</v>
+      </c>
+      <c r="N186" s="4">
+        <v>422.0</v>
+      </c>
+      <c r="O186" s="4">
+        <v>10.0</v>
+      </c>
+      <c r="P186" s="4">
+        <v>14.0</v>
+      </c>
+      <c r="Q186" s="4">
+        <v>460.0</v>
+      </c>
+      <c r="R186" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="S186" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="T186" s="11"/>
+      <c r="U186" s="11"/>
+      <c r="V186" s="9"/>
+      <c r="W186" s="9"/>
       <c r="X186" s="6"/>
       <c r="Y186" s="6"/>
       <c r="Z186" s="6"/>
@@ -14389,30 +14490,68 @@
       <c r="AE186" s="6"/>
       <c r="AF186" s="6"/>
     </row>
-    <row r="187">
-      <c r="A187" s="12"/>
-      <c r="B187" s="6"/>
-      <c r="C187" s="6"/>
-      <c r="D187" s="6"/>
-      <c r="E187" s="6"/>
-      <c r="F187" s="12"/>
-      <c r="G187" s="12"/>
-      <c r="H187" s="12"/>
-      <c r="I187" s="13"/>
-      <c r="J187" s="13"/>
-      <c r="K187" s="13"/>
-      <c r="L187" s="13"/>
-      <c r="M187" s="13"/>
-      <c r="N187" s="13"/>
-      <c r="O187" s="13"/>
-      <c r="P187" s="13"/>
-      <c r="Q187" s="13"/>
-      <c r="R187" s="6"/>
-      <c r="S187" s="6"/>
-      <c r="T187" s="6"/>
-      <c r="U187" s="6"/>
-      <c r="V187" s="6"/>
-      <c r="W187" s="6"/>
+    <row r="187" ht="22.5" customHeight="1">
+      <c r="A187" s="7" t="s">
+        <v>606</v>
+      </c>
+      <c r="B187" s="8">
+        <v>46210.876747685186</v>
+      </c>
+      <c r="C187" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D187" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E187" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F187" s="10" t="s">
+        <v>594</v>
+      </c>
+      <c r="G187" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H187" s="7" t="s">
+        <v>595</v>
+      </c>
+      <c r="I187" s="3">
+        <v>98.13</v>
+      </c>
+      <c r="J187" s="3">
+        <v>98.11</v>
+      </c>
+      <c r="K187" s="3">
+        <v>98.12</v>
+      </c>
+      <c r="L187" s="3">
+        <v>98.12</v>
+      </c>
+      <c r="M187" s="3">
+        <v>98.38</v>
+      </c>
+      <c r="N187" s="4">
+        <v>425.0</v>
+      </c>
+      <c r="O187" s="4">
+        <v>7.0</v>
+      </c>
+      <c r="P187" s="4">
+        <v>10.0</v>
+      </c>
+      <c r="Q187" s="4">
+        <v>464.0</v>
+      </c>
+      <c r="R187" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="S187" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="T187" s="11"/>
+      <c r="U187" s="11"/>
+      <c r="V187" s="9"/>
+      <c r="W187" s="9"/>
       <c r="X187" s="6"/>
       <c r="Y187" s="6"/>
       <c r="Z187" s="6"/>
@@ -14423,30 +14562,68 @@
       <c r="AE187" s="6"/>
       <c r="AF187" s="6"/>
     </row>
-    <row r="188">
-      <c r="A188" s="12"/>
-      <c r="B188" s="6"/>
-      <c r="C188" s="6"/>
-      <c r="D188" s="6"/>
-      <c r="E188" s="6"/>
-      <c r="F188" s="12"/>
-      <c r="G188" s="12"/>
-      <c r="H188" s="12"/>
-      <c r="I188" s="13"/>
-      <c r="J188" s="13"/>
-      <c r="K188" s="13"/>
-      <c r="L188" s="13"/>
-      <c r="M188" s="13"/>
-      <c r="N188" s="13"/>
-      <c r="O188" s="13"/>
-      <c r="P188" s="13"/>
-      <c r="Q188" s="13"/>
-      <c r="R188" s="6"/>
-      <c r="S188" s="6"/>
-      <c r="T188" s="6"/>
-      <c r="U188" s="6"/>
-      <c r="V188" s="6"/>
-      <c r="W188" s="6"/>
+    <row r="188" ht="22.5" customHeight="1">
+      <c r="A188" s="7" t="s">
+        <v>607</v>
+      </c>
+      <c r="B188" s="8">
+        <v>46210.8775</v>
+      </c>
+      <c r="C188" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D188" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E188" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F188" s="10" t="s">
+        <v>597</v>
+      </c>
+      <c r="G188" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H188" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="I188" s="3">
+        <v>96.92</v>
+      </c>
+      <c r="J188" s="3">
+        <v>96.89</v>
+      </c>
+      <c r="K188" s="3">
+        <v>96.9</v>
+      </c>
+      <c r="L188" s="3">
+        <v>96.91</v>
+      </c>
+      <c r="M188" s="3">
+        <v>97.22</v>
+      </c>
+      <c r="N188" s="4">
+        <v>420.0</v>
+      </c>
+      <c r="O188" s="4">
+        <v>12.0</v>
+      </c>
+      <c r="P188" s="4">
+        <v>16.0</v>
+      </c>
+      <c r="Q188" s="4">
+        <v>458.0</v>
+      </c>
+      <c r="R188" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="S188" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="T188" s="11"/>
+      <c r="U188" s="11"/>
+      <c r="V188" s="9"/>
+      <c r="W188" s="9"/>
       <c r="X188" s="6"/>
       <c r="Y188" s="6"/>
       <c r="Z188" s="6"/>
@@ -14457,30 +14634,68 @@
       <c r="AE188" s="6"/>
       <c r="AF188" s="6"/>
     </row>
-    <row r="189">
-      <c r="A189" s="12"/>
-      <c r="B189" s="6"/>
-      <c r="C189" s="6"/>
-      <c r="D189" s="6"/>
-      <c r="E189" s="6"/>
-      <c r="F189" s="12"/>
-      <c r="G189" s="12"/>
-      <c r="H189" s="12"/>
-      <c r="I189" s="13"/>
-      <c r="J189" s="13"/>
-      <c r="K189" s="13"/>
-      <c r="L189" s="13"/>
-      <c r="M189" s="13"/>
-      <c r="N189" s="13"/>
-      <c r="O189" s="13"/>
-      <c r="P189" s="13"/>
-      <c r="Q189" s="13"/>
-      <c r="R189" s="6"/>
-      <c r="S189" s="6"/>
-      <c r="T189" s="6"/>
-      <c r="U189" s="6"/>
-      <c r="V189" s="6"/>
-      <c r="W189" s="6"/>
+    <row r="189" ht="22.5" customHeight="1">
+      <c r="A189" s="7" t="s">
+        <v>608</v>
+      </c>
+      <c r="B189" s="8">
+        <v>46217.75806712963</v>
+      </c>
+      <c r="C189" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D189" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E189" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F189" s="10" t="s">
+        <v>600</v>
+      </c>
+      <c r="G189" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H189" s="7" t="s">
+        <v>601</v>
+      </c>
+      <c r="I189" s="3">
+        <v>96.02</v>
+      </c>
+      <c r="J189" s="3">
+        <v>96.02</v>
+      </c>
+      <c r="K189" s="3">
+        <v>96.02</v>
+      </c>
+      <c r="L189" s="3">
+        <v>96.03</v>
+      </c>
+      <c r="M189" s="3">
+        <v>95.6</v>
+      </c>
+      <c r="N189" s="4">
+        <v>414.0</v>
+      </c>
+      <c r="O189" s="4">
+        <v>18.0</v>
+      </c>
+      <c r="P189" s="4">
+        <v>18.0</v>
+      </c>
+      <c r="Q189" s="4">
+        <v>456.0</v>
+      </c>
+      <c r="R189" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="S189" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="T189" s="11"/>
+      <c r="U189" s="11"/>
+      <c r="V189" s="9"/>
+      <c r="W189" s="9"/>
       <c r="X189" s="6"/>
       <c r="Y189" s="6"/>
       <c r="Z189" s="6"/>
@@ -14491,30 +14706,68 @@
       <c r="AE189" s="6"/>
       <c r="AF189" s="6"/>
     </row>
-    <row r="190">
-      <c r="A190" s="12"/>
-      <c r="B190" s="6"/>
-      <c r="C190" s="6"/>
-      <c r="D190" s="6"/>
-      <c r="E190" s="6"/>
-      <c r="F190" s="12"/>
-      <c r="G190" s="12"/>
-      <c r="H190" s="12"/>
-      <c r="I190" s="13"/>
-      <c r="J190" s="13"/>
-      <c r="K190" s="13"/>
-      <c r="L190" s="13"/>
-      <c r="M190" s="13"/>
-      <c r="N190" s="13"/>
-      <c r="O190" s="13"/>
-      <c r="P190" s="13"/>
-      <c r="Q190" s="13"/>
-      <c r="R190" s="6"/>
-      <c r="S190" s="6"/>
-      <c r="T190" s="6"/>
-      <c r="U190" s="6"/>
-      <c r="V190" s="6"/>
-      <c r="W190" s="6"/>
+    <row r="190" ht="22.5" customHeight="1">
+      <c r="A190" s="7" t="s">
+        <v>609</v>
+      </c>
+      <c r="B190" s="8">
+        <v>46217.76155092593</v>
+      </c>
+      <c r="C190" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D190" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E190" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F190" s="10" t="s">
+        <v>603</v>
+      </c>
+      <c r="G190" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H190" s="7" t="s">
+        <v>604</v>
+      </c>
+      <c r="I190" s="3">
+        <v>96.01</v>
+      </c>
+      <c r="J190" s="3">
+        <v>96.03</v>
+      </c>
+      <c r="K190" s="3">
+        <v>96.02</v>
+      </c>
+      <c r="L190" s="3">
+        <v>96.03</v>
+      </c>
+      <c r="M190" s="3">
+        <v>95.37</v>
+      </c>
+      <c r="N190" s="4">
+        <v>413.0</v>
+      </c>
+      <c r="O190" s="4">
+        <v>19.0</v>
+      </c>
+      <c r="P190" s="4">
+        <v>17.0</v>
+      </c>
+      <c r="Q190" s="4">
+        <v>457.0</v>
+      </c>
+      <c r="R190" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="S190" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="T190" s="11"/>
+      <c r="U190" s="11"/>
+      <c r="V190" s="9"/>
+      <c r="W190" s="9"/>
       <c r="X190" s="6"/>
       <c r="Y190" s="6"/>
       <c r="Z190" s="6"/>
@@ -14525,30 +14778,68 @@
       <c r="AE190" s="6"/>
       <c r="AF190" s="6"/>
     </row>
-    <row r="191">
-      <c r="A191" s="12"/>
-      <c r="B191" s="6"/>
-      <c r="C191" s="6"/>
-      <c r="D191" s="6"/>
-      <c r="E191" s="6"/>
-      <c r="F191" s="12"/>
-      <c r="G191" s="12"/>
-      <c r="H191" s="12"/>
-      <c r="I191" s="13"/>
-      <c r="J191" s="13"/>
-      <c r="K191" s="13"/>
-      <c r="L191" s="13"/>
-      <c r="M191" s="13"/>
-      <c r="N191" s="13"/>
-      <c r="O191" s="13"/>
-      <c r="P191" s="13"/>
-      <c r="Q191" s="13"/>
-      <c r="R191" s="6"/>
-      <c r="S191" s="6"/>
-      <c r="T191" s="6"/>
-      <c r="U191" s="6"/>
-      <c r="V191" s="6"/>
-      <c r="W191" s="6"/>
+    <row r="191" ht="22.5" customHeight="1">
+      <c r="A191" s="7" t="s">
+        <v>610</v>
+      </c>
+      <c r="B191" s="8">
+        <v>46236.8549537037</v>
+      </c>
+      <c r="C191" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D191" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E191" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F191" s="10" t="s">
+        <v>611</v>
+      </c>
+      <c r="G191" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H191" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="I191" s="3">
+        <v>98.02</v>
+      </c>
+      <c r="J191" s="3">
+        <v>98.0</v>
+      </c>
+      <c r="K191" s="3">
+        <v>98.01</v>
+      </c>
+      <c r="L191" s="3">
+        <v>98.01</v>
+      </c>
+      <c r="M191" s="3">
+        <v>98.15</v>
+      </c>
+      <c r="N191" s="4">
+        <v>424.0</v>
+      </c>
+      <c r="O191" s="4">
+        <v>8.0</v>
+      </c>
+      <c r="P191" s="4">
+        <v>10.0</v>
+      </c>
+      <c r="Q191" s="4">
+        <v>464.0</v>
+      </c>
+      <c r="R191" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="S191" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="T191" s="11"/>
+      <c r="U191" s="11"/>
+      <c r="V191" s="9"/>
+      <c r="W191" s="9"/>
       <c r="X191" s="6"/>
       <c r="Y191" s="6"/>
       <c r="Z191" s="6"/>
@@ -14559,30 +14850,68 @@
       <c r="AE191" s="6"/>
       <c r="AF191" s="6"/>
     </row>
-    <row r="192">
-      <c r="A192" s="12"/>
-      <c r="B192" s="6"/>
-      <c r="C192" s="6"/>
-      <c r="D192" s="6"/>
-      <c r="E192" s="6"/>
-      <c r="F192" s="12"/>
-      <c r="G192" s="12"/>
-      <c r="H192" s="12"/>
-      <c r="I192" s="13"/>
-      <c r="J192" s="13"/>
-      <c r="K192" s="13"/>
-      <c r="L192" s="13"/>
-      <c r="M192" s="13"/>
-      <c r="N192" s="13"/>
-      <c r="O192" s="13"/>
-      <c r="P192" s="13"/>
-      <c r="Q192" s="13"/>
-      <c r="R192" s="6"/>
-      <c r="S192" s="6"/>
-      <c r="T192" s="6"/>
-      <c r="U192" s="6"/>
-      <c r="V192" s="6"/>
-      <c r="W192" s="6"/>
+    <row r="192" ht="22.5" customHeight="1">
+      <c r="A192" s="7" t="s">
+        <v>613</v>
+      </c>
+      <c r="B192" s="8">
+        <v>46236.85621527778</v>
+      </c>
+      <c r="C192" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D192" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E192" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F192" s="10" t="s">
+        <v>614</v>
+      </c>
+      <c r="G192" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H192" s="7" t="s">
+        <v>615</v>
+      </c>
+      <c r="I192" s="3">
+        <v>97.25</v>
+      </c>
+      <c r="J192" s="3">
+        <v>97.22</v>
+      </c>
+      <c r="K192" s="3">
+        <v>97.24</v>
+      </c>
+      <c r="L192" s="3">
+        <v>97.24</v>
+      </c>
+      <c r="M192" s="3">
+        <v>97.45</v>
+      </c>
+      <c r="N192" s="4">
+        <v>421.0</v>
+      </c>
+      <c r="O192" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="P192" s="4">
+        <v>14.0</v>
+      </c>
+      <c r="Q192" s="4">
+        <v>460.0</v>
+      </c>
+      <c r="R192" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="S192" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="T192" s="11"/>
+      <c r="U192" s="11"/>
+      <c r="V192" s="9"/>
+      <c r="W192" s="9"/>
       <c r="X192" s="6"/>
       <c r="Y192" s="6"/>
       <c r="Z192" s="6"/>
@@ -14593,30 +14922,68 @@
       <c r="AE192" s="6"/>
       <c r="AF192" s="6"/>
     </row>
-    <row r="193">
-      <c r="A193" s="12"/>
-      <c r="B193" s="6"/>
-      <c r="C193" s="6"/>
-      <c r="D193" s="6"/>
-      <c r="E193" s="6"/>
-      <c r="F193" s="12"/>
-      <c r="G193" s="12"/>
-      <c r="H193" s="12"/>
-      <c r="I193" s="13"/>
-      <c r="J193" s="13"/>
-      <c r="K193" s="13"/>
-      <c r="L193" s="13"/>
-      <c r="M193" s="13"/>
-      <c r="N193" s="13"/>
-      <c r="O193" s="13"/>
-      <c r="P193" s="13"/>
-      <c r="Q193" s="13"/>
-      <c r="R193" s="6"/>
-      <c r="S193" s="6"/>
-      <c r="T193" s="6"/>
-      <c r="U193" s="6"/>
-      <c r="V193" s="6"/>
-      <c r="W193" s="6"/>
+    <row r="193" ht="22.5" customHeight="1">
+      <c r="A193" s="7" t="s">
+        <v>616</v>
+      </c>
+      <c r="B193" s="8">
+        <v>46236.85738425926</v>
+      </c>
+      <c r="C193" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D193" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E193" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F193" s="10" t="s">
+        <v>617</v>
+      </c>
+      <c r="G193" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H193" s="7" t="s">
+        <v>618</v>
+      </c>
+      <c r="I193" s="3">
+        <v>97.47</v>
+      </c>
+      <c r="J193" s="3">
+        <v>97.44</v>
+      </c>
+      <c r="K193" s="3">
+        <v>97.46</v>
+      </c>
+      <c r="L193" s="3">
+        <v>97.46</v>
+      </c>
+      <c r="M193" s="3">
+        <v>97.69</v>
+      </c>
+      <c r="N193" s="4">
+        <v>422.0</v>
+      </c>
+      <c r="O193" s="4">
+        <v>10.0</v>
+      </c>
+      <c r="P193" s="4">
+        <v>13.0</v>
+      </c>
+      <c r="Q193" s="4">
+        <v>461.0</v>
+      </c>
+      <c r="R193" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="S193" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="T193" s="11"/>
+      <c r="U193" s="11"/>
+      <c r="V193" s="9"/>
+      <c r="W193" s="9"/>
       <c r="X193" s="6"/>
       <c r="Y193" s="6"/>
       <c r="Z193" s="6"/>
@@ -14627,30 +14994,68 @@
       <c r="AE193" s="6"/>
       <c r="AF193" s="6"/>
     </row>
-    <row r="194">
-      <c r="A194" s="12"/>
-      <c r="B194" s="6"/>
-      <c r="C194" s="6"/>
-      <c r="D194" s="6"/>
-      <c r="E194" s="6"/>
-      <c r="F194" s="12"/>
-      <c r="G194" s="12"/>
-      <c r="H194" s="12"/>
-      <c r="I194" s="13"/>
-      <c r="J194" s="13"/>
-      <c r="K194" s="13"/>
-      <c r="L194" s="13"/>
-      <c r="M194" s="13"/>
-      <c r="N194" s="13"/>
-      <c r="O194" s="13"/>
-      <c r="P194" s="13"/>
-      <c r="Q194" s="13"/>
-      <c r="R194" s="6"/>
-      <c r="S194" s="6"/>
-      <c r="T194" s="6"/>
-      <c r="U194" s="6"/>
-      <c r="V194" s="6"/>
-      <c r="W194" s="6"/>
+    <row r="194" ht="22.5" customHeight="1">
+      <c r="A194" s="7" t="s">
+        <v>619</v>
+      </c>
+      <c r="B194" s="8">
+        <v>46236.88182870371</v>
+      </c>
+      <c r="C194" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D194" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E194" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F194" s="10" t="s">
+        <v>620</v>
+      </c>
+      <c r="G194" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H194" s="7" t="s">
+        <v>621</v>
+      </c>
+      <c r="I194" s="3">
+        <v>95.15</v>
+      </c>
+      <c r="J194" s="3">
+        <v>95.12</v>
+      </c>
+      <c r="K194" s="3">
+        <v>95.13</v>
+      </c>
+      <c r="L194" s="3">
+        <v>95.14</v>
+      </c>
+      <c r="M194" s="3">
+        <v>95.37</v>
+      </c>
+      <c r="N194" s="4">
+        <v>412.0</v>
+      </c>
+      <c r="O194" s="4">
+        <v>20.0</v>
+      </c>
+      <c r="P194" s="4">
+        <v>24.0</v>
+      </c>
+      <c r="Q194" s="4">
+        <v>450.0</v>
+      </c>
+      <c r="R194" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="S194" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="T194" s="11"/>
+      <c r="U194" s="11"/>
+      <c r="V194" s="9"/>
+      <c r="W194" s="9"/>
       <c r="X194" s="6"/>
       <c r="Y194" s="6"/>
       <c r="Z194" s="6"/>
@@ -14661,30 +15066,68 @@
       <c r="AE194" s="6"/>
       <c r="AF194" s="6"/>
     </row>
-    <row r="195">
-      <c r="A195" s="12"/>
-      <c r="B195" s="6"/>
-      <c r="C195" s="6"/>
-      <c r="D195" s="6"/>
-      <c r="E195" s="6"/>
-      <c r="F195" s="12"/>
-      <c r="G195" s="12"/>
-      <c r="H195" s="12"/>
-      <c r="I195" s="13"/>
-      <c r="J195" s="13"/>
-      <c r="K195" s="13"/>
-      <c r="L195" s="13"/>
-      <c r="M195" s="13"/>
-      <c r="N195" s="13"/>
-      <c r="O195" s="13"/>
-      <c r="P195" s="13"/>
-      <c r="Q195" s="13"/>
-      <c r="R195" s="6"/>
-      <c r="S195" s="6"/>
-      <c r="T195" s="6"/>
-      <c r="U195" s="6"/>
-      <c r="V195" s="6"/>
-      <c r="W195" s="6"/>
+    <row r="195" ht="22.5" customHeight="1">
+      <c r="A195" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="B195" s="8">
+        <v>46236.88282407408</v>
+      </c>
+      <c r="C195" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D195" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E195" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F195" s="10" t="s">
+        <v>623</v>
+      </c>
+      <c r="G195" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H195" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="I195" s="3">
+        <v>97.8</v>
+      </c>
+      <c r="J195" s="3">
+        <v>97.78</v>
+      </c>
+      <c r="K195" s="3">
+        <v>97.79</v>
+      </c>
+      <c r="L195" s="3">
+        <v>97.79</v>
+      </c>
+      <c r="M195" s="3">
+        <v>97.92</v>
+      </c>
+      <c r="N195" s="4">
+        <v>423.0</v>
+      </c>
+      <c r="O195" s="4">
+        <v>9.0</v>
+      </c>
+      <c r="P195" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="Q195" s="4">
+        <v>463.0</v>
+      </c>
+      <c r="R195" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="S195" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="T195" s="11"/>
+      <c r="U195" s="11"/>
+      <c r="V195" s="9"/>
+      <c r="W195" s="9"/>
       <c r="X195" s="6"/>
       <c r="Y195" s="6"/>
       <c r="Z195" s="6"/>
@@ -48456,6 +48899,346 @@
       <c r="AD1188" s="6"/>
       <c r="AE1188" s="6"/>
       <c r="AF1188" s="6"/>
+    </row>
+    <row r="1189">
+      <c r="A1189" s="12"/>
+      <c r="B1189" s="6"/>
+      <c r="C1189" s="6"/>
+      <c r="D1189" s="6"/>
+      <c r="E1189" s="6"/>
+      <c r="F1189" s="12"/>
+      <c r="G1189" s="12"/>
+      <c r="H1189" s="12"/>
+      <c r="I1189" s="13"/>
+      <c r="J1189" s="13"/>
+      <c r="K1189" s="13"/>
+      <c r="L1189" s="13"/>
+      <c r="M1189" s="13"/>
+      <c r="N1189" s="13"/>
+      <c r="O1189" s="13"/>
+      <c r="P1189" s="13"/>
+      <c r="Q1189" s="13"/>
+      <c r="R1189" s="6"/>
+      <c r="S1189" s="6"/>
+      <c r="T1189" s="6"/>
+      <c r="U1189" s="6"/>
+      <c r="V1189" s="6"/>
+      <c r="W1189" s="6"/>
+      <c r="X1189" s="6"/>
+      <c r="Y1189" s="6"/>
+      <c r="Z1189" s="6"/>
+      <c r="AA1189" s="6"/>
+      <c r="AB1189" s="6"/>
+      <c r="AC1189" s="6"/>
+      <c r="AD1189" s="6"/>
+      <c r="AE1189" s="6"/>
+      <c r="AF1189" s="6"/>
+    </row>
+    <row r="1190">
+      <c r="A1190" s="12"/>
+      <c r="B1190" s="6"/>
+      <c r="C1190" s="6"/>
+      <c r="D1190" s="6"/>
+      <c r="E1190" s="6"/>
+      <c r="F1190" s="12"/>
+      <c r="G1190" s="12"/>
+      <c r="H1190" s="12"/>
+      <c r="I1190" s="13"/>
+      <c r="J1190" s="13"/>
+      <c r="K1190" s="13"/>
+      <c r="L1190" s="13"/>
+      <c r="M1190" s="13"/>
+      <c r="N1190" s="13"/>
+      <c r="O1190" s="13"/>
+      <c r="P1190" s="13"/>
+      <c r="Q1190" s="13"/>
+      <c r="R1190" s="6"/>
+      <c r="S1190" s="6"/>
+      <c r="T1190" s="6"/>
+      <c r="U1190" s="6"/>
+      <c r="V1190" s="6"/>
+      <c r="W1190" s="6"/>
+      <c r="X1190" s="6"/>
+      <c r="Y1190" s="6"/>
+      <c r="Z1190" s="6"/>
+      <c r="AA1190" s="6"/>
+      <c r="AB1190" s="6"/>
+      <c r="AC1190" s="6"/>
+      <c r="AD1190" s="6"/>
+      <c r="AE1190" s="6"/>
+      <c r="AF1190" s="6"/>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="12"/>
+      <c r="B1191" s="6"/>
+      <c r="C1191" s="6"/>
+      <c r="D1191" s="6"/>
+      <c r="E1191" s="6"/>
+      <c r="F1191" s="12"/>
+      <c r="G1191" s="12"/>
+      <c r="H1191" s="12"/>
+      <c r="I1191" s="13"/>
+      <c r="J1191" s="13"/>
+      <c r="K1191" s="13"/>
+      <c r="L1191" s="13"/>
+      <c r="M1191" s="13"/>
+      <c r="N1191" s="13"/>
+      <c r="O1191" s="13"/>
+      <c r="P1191" s="13"/>
+      <c r="Q1191" s="13"/>
+      <c r="R1191" s="6"/>
+      <c r="S1191" s="6"/>
+      <c r="T1191" s="6"/>
+      <c r="U1191" s="6"/>
+      <c r="V1191" s="6"/>
+      <c r="W1191" s="6"/>
+      <c r="X1191" s="6"/>
+      <c r="Y1191" s="6"/>
+      <c r="Z1191" s="6"/>
+      <c r="AA1191" s="6"/>
+      <c r="AB1191" s="6"/>
+      <c r="AC1191" s="6"/>
+      <c r="AD1191" s="6"/>
+      <c r="AE1191" s="6"/>
+      <c r="AF1191" s="6"/>
+    </row>
+    <row r="1192">
+      <c r="A1192" s="12"/>
+      <c r="B1192" s="6"/>
+      <c r="C1192" s="6"/>
+      <c r="D1192" s="6"/>
+      <c r="E1192" s="6"/>
+      <c r="F1192" s="12"/>
+      <c r="G1192" s="12"/>
+      <c r="H1192" s="12"/>
+      <c r="I1192" s="13"/>
+      <c r="J1192" s="13"/>
+      <c r="K1192" s="13"/>
+      <c r="L1192" s="13"/>
+      <c r="M1192" s="13"/>
+      <c r="N1192" s="13"/>
+      <c r="O1192" s="13"/>
+      <c r="P1192" s="13"/>
+      <c r="Q1192" s="13"/>
+      <c r="R1192" s="6"/>
+      <c r="S1192" s="6"/>
+      <c r="T1192" s="6"/>
+      <c r="U1192" s="6"/>
+      <c r="V1192" s="6"/>
+      <c r="W1192" s="6"/>
+      <c r="X1192" s="6"/>
+      <c r="Y1192" s="6"/>
+      <c r="Z1192" s="6"/>
+      <c r="AA1192" s="6"/>
+      <c r="AB1192" s="6"/>
+      <c r="AC1192" s="6"/>
+      <c r="AD1192" s="6"/>
+      <c r="AE1192" s="6"/>
+      <c r="AF1192" s="6"/>
+    </row>
+    <row r="1193">
+      <c r="A1193" s="12"/>
+      <c r="B1193" s="6"/>
+      <c r="C1193" s="6"/>
+      <c r="D1193" s="6"/>
+      <c r="E1193" s="6"/>
+      <c r="F1193" s="12"/>
+      <c r="G1193" s="12"/>
+      <c r="H1193" s="12"/>
+      <c r="I1193" s="13"/>
+      <c r="J1193" s="13"/>
+      <c r="K1193" s="13"/>
+      <c r="L1193" s="13"/>
+      <c r="M1193" s="13"/>
+      <c r="N1193" s="13"/>
+      <c r="O1193" s="13"/>
+      <c r="P1193" s="13"/>
+      <c r="Q1193" s="13"/>
+      <c r="R1193" s="6"/>
+      <c r="S1193" s="6"/>
+      <c r="T1193" s="6"/>
+      <c r="U1193" s="6"/>
+      <c r="V1193" s="6"/>
+      <c r="W1193" s="6"/>
+      <c r="X1193" s="6"/>
+      <c r="Y1193" s="6"/>
+      <c r="Z1193" s="6"/>
+      <c r="AA1193" s="6"/>
+      <c r="AB1193" s="6"/>
+      <c r="AC1193" s="6"/>
+      <c r="AD1193" s="6"/>
+      <c r="AE1193" s="6"/>
+      <c r="AF1193" s="6"/>
+    </row>
+    <row r="1194">
+      <c r="A1194" s="12"/>
+      <c r="B1194" s="6"/>
+      <c r="C1194" s="6"/>
+      <c r="D1194" s="6"/>
+      <c r="E1194" s="6"/>
+      <c r="F1194" s="12"/>
+      <c r="G1194" s="12"/>
+      <c r="H1194" s="12"/>
+      <c r="I1194" s="13"/>
+      <c r="J1194" s="13"/>
+      <c r="K1194" s="13"/>
+      <c r="L1194" s="13"/>
+      <c r="M1194" s="13"/>
+      <c r="N1194" s="13"/>
+      <c r="O1194" s="13"/>
+      <c r="P1194" s="13"/>
+      <c r="Q1194" s="13"/>
+      <c r="R1194" s="6"/>
+      <c r="S1194" s="6"/>
+      <c r="T1194" s="6"/>
+      <c r="U1194" s="6"/>
+      <c r="V1194" s="6"/>
+      <c r="W1194" s="6"/>
+      <c r="X1194" s="6"/>
+      <c r="Y1194" s="6"/>
+      <c r="Z1194" s="6"/>
+      <c r="AA1194" s="6"/>
+      <c r="AB1194" s="6"/>
+      <c r="AC1194" s="6"/>
+      <c r="AD1194" s="6"/>
+      <c r="AE1194" s="6"/>
+      <c r="AF1194" s="6"/>
+    </row>
+    <row r="1195">
+      <c r="A1195" s="12"/>
+      <c r="B1195" s="6"/>
+      <c r="C1195" s="6"/>
+      <c r="D1195" s="6"/>
+      <c r="E1195" s="6"/>
+      <c r="F1195" s="12"/>
+      <c r="G1195" s="12"/>
+      <c r="H1195" s="12"/>
+      <c r="I1195" s="13"/>
+      <c r="J1195" s="13"/>
+      <c r="K1195" s="13"/>
+      <c r="L1195" s="13"/>
+      <c r="M1195" s="13"/>
+      <c r="N1195" s="13"/>
+      <c r="O1195" s="13"/>
+      <c r="P1195" s="13"/>
+      <c r="Q1195" s="13"/>
+      <c r="R1195" s="6"/>
+      <c r="S1195" s="6"/>
+      <c r="T1195" s="6"/>
+      <c r="U1195" s="6"/>
+      <c r="V1195" s="6"/>
+      <c r="W1195" s="6"/>
+      <c r="X1195" s="6"/>
+      <c r="Y1195" s="6"/>
+      <c r="Z1195" s="6"/>
+      <c r="AA1195" s="6"/>
+      <c r="AB1195" s="6"/>
+      <c r="AC1195" s="6"/>
+      <c r="AD1195" s="6"/>
+      <c r="AE1195" s="6"/>
+      <c r="AF1195" s="6"/>
+    </row>
+    <row r="1196">
+      <c r="A1196" s="12"/>
+      <c r="B1196" s="6"/>
+      <c r="C1196" s="6"/>
+      <c r="D1196" s="6"/>
+      <c r="E1196" s="6"/>
+      <c r="F1196" s="12"/>
+      <c r="G1196" s="12"/>
+      <c r="H1196" s="12"/>
+      <c r="I1196" s="13"/>
+      <c r="J1196" s="13"/>
+      <c r="K1196" s="13"/>
+      <c r="L1196" s="13"/>
+      <c r="M1196" s="13"/>
+      <c r="N1196" s="13"/>
+      <c r="O1196" s="13"/>
+      <c r="P1196" s="13"/>
+      <c r="Q1196" s="13"/>
+      <c r="R1196" s="6"/>
+      <c r="S1196" s="6"/>
+      <c r="T1196" s="6"/>
+      <c r="U1196" s="6"/>
+      <c r="V1196" s="6"/>
+      <c r="W1196" s="6"/>
+      <c r="X1196" s="6"/>
+      <c r="Y1196" s="6"/>
+      <c r="Z1196" s="6"/>
+      <c r="AA1196" s="6"/>
+      <c r="AB1196" s="6"/>
+      <c r="AC1196" s="6"/>
+      <c r="AD1196" s="6"/>
+      <c r="AE1196" s="6"/>
+      <c r="AF1196" s="6"/>
+    </row>
+    <row r="1197">
+      <c r="A1197" s="12"/>
+      <c r="B1197" s="6"/>
+      <c r="C1197" s="6"/>
+      <c r="D1197" s="6"/>
+      <c r="E1197" s="6"/>
+      <c r="F1197" s="12"/>
+      <c r="G1197" s="12"/>
+      <c r="H1197" s="12"/>
+      <c r="I1197" s="13"/>
+      <c r="J1197" s="13"/>
+      <c r="K1197" s="13"/>
+      <c r="L1197" s="13"/>
+      <c r="M1197" s="13"/>
+      <c r="N1197" s="13"/>
+      <c r="O1197" s="13"/>
+      <c r="P1197" s="13"/>
+      <c r="Q1197" s="13"/>
+      <c r="R1197" s="6"/>
+      <c r="S1197" s="6"/>
+      <c r="T1197" s="6"/>
+      <c r="U1197" s="6"/>
+      <c r="V1197" s="6"/>
+      <c r="W1197" s="6"/>
+      <c r="X1197" s="6"/>
+      <c r="Y1197" s="6"/>
+      <c r="Z1197" s="6"/>
+      <c r="AA1197" s="6"/>
+      <c r="AB1197" s="6"/>
+      <c r="AC1197" s="6"/>
+      <c r="AD1197" s="6"/>
+      <c r="AE1197" s="6"/>
+      <c r="AF1197" s="6"/>
+    </row>
+    <row r="1198">
+      <c r="A1198" s="12"/>
+      <c r="B1198" s="6"/>
+      <c r="C1198" s="6"/>
+      <c r="D1198" s="6"/>
+      <c r="E1198" s="6"/>
+      <c r="F1198" s="12"/>
+      <c r="G1198" s="12"/>
+      <c r="H1198" s="12"/>
+      <c r="I1198" s="13"/>
+      <c r="J1198" s="13"/>
+      <c r="K1198" s="13"/>
+      <c r="L1198" s="13"/>
+      <c r="M1198" s="13"/>
+      <c r="N1198" s="13"/>
+      <c r="O1198" s="13"/>
+      <c r="P1198" s="13"/>
+      <c r="Q1198" s="13"/>
+      <c r="R1198" s="6"/>
+      <c r="S1198" s="6"/>
+      <c r="T1198" s="6"/>
+      <c r="U1198" s="6"/>
+      <c r="V1198" s="6"/>
+      <c r="W1198" s="6"/>
+      <c r="X1198" s="6"/>
+      <c r="Y1198" s="6"/>
+      <c r="Z1198" s="6"/>
+      <c r="AA1198" s="6"/>
+      <c r="AB1198" s="6"/>
+      <c r="AC1198" s="6"/>
+      <c r="AD1198" s="6"/>
+      <c r="AE1198" s="6"/>
+      <c r="AF1198" s="6"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -48643,10 +49426,20 @@
     <hyperlink r:id="rId182" ref="F183"/>
     <hyperlink r:id="rId183" ref="F184"/>
     <hyperlink r:id="rId184" ref="F185"/>
+    <hyperlink r:id="rId185" ref="F186"/>
+    <hyperlink r:id="rId186" ref="F187"/>
+    <hyperlink r:id="rId187" ref="F188"/>
+    <hyperlink r:id="rId188" ref="F189"/>
+    <hyperlink r:id="rId189" ref="F190"/>
+    <hyperlink r:id="rId190" ref="F191"/>
+    <hyperlink r:id="rId191" ref="F192"/>
+    <hyperlink r:id="rId192" ref="F193"/>
+    <hyperlink r:id="rId193" ref="F194"/>
+    <hyperlink r:id="rId194" ref="F195"/>
   </hyperlinks>
-  <drawing r:id="rId185"/>
+  <drawing r:id="rId195"/>
   <tableParts count="1">
-    <tablePart r:id="rId187"/>
+    <tablePart r:id="rId197"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updating ProvideQ run label
</commit_message>
<xml_diff>
--- a/assets/SciClaimEval26_Results.xlsx
+++ b/assets/SciClaimEval26_Results.xlsx
@@ -2292,7 +2292,7 @@
     <col customWidth="1" min="1" max="1" width="8.75"/>
     <col customWidth="1" min="2" max="2" width="17.13"/>
     <col customWidth="1" min="4" max="4" width="14.75"/>
-    <col customWidth="1" min="6" max="6" width="10.13"/>
+    <col customWidth="1" min="6" max="6" width="61.25"/>
     <col customWidth="1" min="7" max="7" width="12.5"/>
     <col customWidth="1" min="8" max="8" width="30.13"/>
     <col customWidth="1" min="9" max="9" width="9.75"/>
@@ -10010,7 +10010,7 @@
         <v>392</v>
       </c>
       <c r="G120" s="9" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="H120" s="7" t="s">
         <v>393</v>

</xml_diff>